<commit_message>
Satni obracun: prvo ispravno citanje u satu, obracun i u 01:xx, rezerva ne cita u prvih 10 min
- satno.py: za svaki smer se u satu uzima prvo ISPRAVNO citanje (zakasnela rezerva u 08:00 sa
  brojacem od 07:53 je kvarila sate 8 i 9 dana 10.10.)
- workflow: obracun za juce i u citanju u 01:xx (u 00:02 brojac je cesto jos od 23:58, pa sat 23-24
  dobija "juce" tek u 01:02)
- citaj.py --samo-ako-nema: ne cita u prvih 10 min sata
- ponovo izracunati 09.-11.10. i Excel (10. i 11.10. sada potpuni: 1104/1104 sati)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjLihUGrpExWnzAPATqsnz
</commit_message>
<xml_diff>
--- a/podaci/excel/bicikli_2026-10.xlsx
+++ b/podaci/excel/bicikli_2026-10.xlsx
@@ -1,59 +1,59 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="15a" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="15b" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="20a" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="20b" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="22a" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="22b" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="23a" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="25a" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="26" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="27a" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="27b" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="28" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="29a" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="29b" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="30a" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="30b" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="31b" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="34a" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="34b" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="36a" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="36b" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="37a" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="38a" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="38b" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="39a" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="39b" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="40a" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="40b" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="41" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="42a" sheetId="30" state="visible" r:id="rId30"/>
-    <sheet name="42b" sheetId="31" state="visible" r:id="rId31"/>
-    <sheet name="43a" sheetId="32" state="visible" r:id="rId32"/>
-    <sheet name="43b" sheetId="33" state="visible" r:id="rId33"/>
-    <sheet name="44a" sheetId="34" state="visible" r:id="rId34"/>
-    <sheet name="44b" sheetId="35" state="visible" r:id="rId35"/>
-    <sheet name="45a" sheetId="36" state="visible" r:id="rId36"/>
-    <sheet name="45b" sheetId="37" state="visible" r:id="rId37"/>
-    <sheet name="46a" sheetId="38" state="visible" r:id="rId38"/>
-    <sheet name="46b" sheetId="39" state="visible" r:id="rId39"/>
-    <sheet name="47" sheetId="40" state="visible" r:id="rId40"/>
-    <sheet name="49a" sheetId="41" state="visible" r:id="rId41"/>
-    <sheet name="49b" sheetId="42" state="visible" r:id="rId42"/>
-    <sheet name="50a" sheetId="43" state="visible" r:id="rId43"/>
-    <sheet name="50b" sheetId="44" state="visible" r:id="rId44"/>
-    <sheet name="51a" sheetId="45" state="visible" r:id="rId45"/>
-    <sheet name="51b" sheetId="46" state="visible" r:id="rId46"/>
-    <sheet name="Info" sheetId="47" state="visible" r:id="rId47"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15a" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15b" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20a" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20b" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22a" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="22b" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="23a" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="25a" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="26" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27a" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="27b" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="28" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="29a" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="29b" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30a" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="30b" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="31b" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34a" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="34b" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="36a" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="36b" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="37a" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="38a" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="38b" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="39a" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="39b" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40a" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="40b" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="41" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="42a" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="42b" sheetId="31" state="visible" r:id="rId31"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="43a" sheetId="32" state="visible" r:id="rId32"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="43b" sheetId="33" state="visible" r:id="rId33"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="44a" sheetId="34" state="visible" r:id="rId34"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="44b" sheetId="35" state="visible" r:id="rId35"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="45a" sheetId="36" state="visible" r:id="rId36"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="45b" sheetId="37" state="visible" r:id="rId37"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="46a" sheetId="38" state="visible" r:id="rId38"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="46b" sheetId="39" state="visible" r:id="rId39"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="47" sheetId="40" state="visible" r:id="rId40"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="49a" sheetId="41" state="visible" r:id="rId41"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="49b" sheetId="42" state="visible" r:id="rId42"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50a" sheetId="43" state="visible" r:id="rId43"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="50b" sheetId="44" state="visible" r:id="rId44"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="51a" sheetId="45" state="visible" r:id="rId45"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="51b" sheetId="46" state="visible" r:id="rId46"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="47" state="visible" r:id="rId47"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -975,10 +975,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="34">
@@ -990,10 +989,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="35">
@@ -1201,10 +1199,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -2047,10 +2044,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="34">
@@ -2062,10 +2058,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="35">
@@ -2273,10 +2268,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -3119,10 +3113,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="34">
@@ -3134,10 +3127,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="35">
@@ -3345,10 +3337,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="50">
@@ -4291,10 +4282,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>18</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="34">
@@ -4306,10 +4302,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>33</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="35">
@@ -4601,10 +4602,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>14</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="50">
@@ -5591,10 +5597,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="34">
@@ -5606,10 +5611,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="35">
@@ -5817,10 +5821,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="50">
@@ -6663,10 +6666,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="34">
@@ -6678,10 +6680,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="35">
@@ -6889,10 +6890,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -7735,10 +7735,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="34">
@@ -7750,10 +7749,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="35">
@@ -7961,10 +7959,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="50">
@@ -8807,10 +8804,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="34">
@@ -8822,10 +8818,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="35">
@@ -9033,10 +9028,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -9879,10 +9873,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="34">
@@ -9894,10 +9887,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="35">
@@ -10105,10 +10097,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="50">
@@ -10951,10 +10942,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>68</v>
       </c>
     </row>
     <row r="34">
@@ -10966,10 +10956,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>93</v>
       </c>
     </row>
     <row r="35">
@@ -11177,10 +11166,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="50">
@@ -12023,10 +12011,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="34">
@@ -12038,10 +12025,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>40</v>
       </c>
     </row>
     <row r="35">
@@ -12249,10 +12235,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="50">
@@ -13095,10 +13080,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="34">
@@ -13110,10 +13094,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>36</v>
       </c>
     </row>
     <row r="35">
@@ -13321,10 +13304,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="50">
@@ -14167,10 +14149,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="34">
@@ -14182,10 +14163,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="35">
@@ -14393,10 +14373,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="50">
@@ -15239,10 +15218,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="34">
@@ -15254,10 +15232,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="35">
@@ -15465,10 +15442,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -16311,10 +16287,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="34">
@@ -16326,10 +16301,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="35">
@@ -16537,10 +16511,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -17383,10 +17356,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="34">
@@ -17398,10 +17370,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="35">
@@ -17609,10 +17580,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="50">
@@ -18455,10 +18425,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="34">
@@ -18470,10 +18439,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="35">
@@ -18681,10 +18649,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="50">
@@ -19527,10 +19494,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="34">
@@ -19542,10 +19508,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="35">
@@ -19753,10 +19718,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="50">
@@ -20599,10 +20563,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="34">
@@ -20614,10 +20577,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="35">
@@ -20825,10 +20787,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -21771,10 +21732,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>13</v>
+      </c>
+      <c r="E33" t="n">
+        <v>11</v>
+      </c>
+      <c r="F33" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="34">
@@ -21786,10 +21752,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>23</v>
+      </c>
+      <c r="E34" t="n">
+        <v>9</v>
+      </c>
+      <c r="F34" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="35">
@@ -22081,10 +22052,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="50">
@@ -23171,10 +23147,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>4</v>
+      </c>
+      <c r="E33" t="n">
+        <v>7</v>
+      </c>
+      <c r="F33" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="34">
@@ -23186,10 +23167,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>6</v>
+      </c>
+      <c r="E34" t="n">
+        <v>11</v>
+      </c>
+      <c r="F34" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="35">
@@ -23481,10 +23467,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="50">
@@ -24571,10 +24562,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>28</v>
+      </c>
+      <c r="E33" t="n">
+        <v>14</v>
+      </c>
+      <c r="F33" t="n">
+        <v>42</v>
       </c>
     </row>
     <row r="34">
@@ -24586,10 +24582,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>31</v>
+      </c>
+      <c r="E34" t="n">
+        <v>20</v>
+      </c>
+      <c r="F34" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="35">
@@ -24881,10 +24882,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -25871,10 +25877,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="34">
@@ -25886,10 +25891,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="35">
@@ -26097,10 +26101,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -26943,10 +26946,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -26958,10 +26960,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -27169,10 +27170,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -28015,10 +28015,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="34">
@@ -28030,10 +28029,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="35">
@@ -28241,10 +28239,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="50">
@@ -29087,10 +29084,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="34">
@@ -29102,10 +29098,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="35">
@@ -29313,10 +29308,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -30159,10 +30153,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="34">
@@ -30174,10 +30167,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="35">
@@ -30385,10 +30377,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -31231,10 +31222,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="34">
@@ -31246,10 +31236,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="35">
@@ -31457,10 +31446,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -32303,10 +32291,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="34">
@@ -32318,10 +32305,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="35">
@@ -32529,10 +32515,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="50">
@@ -33375,10 +33360,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="34">
@@ -33390,10 +33374,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="35">
@@ -33601,10 +33584,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -34447,10 +34429,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="34">
@@ -34462,10 +34443,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>27</v>
       </c>
     </row>
     <row r="35">
@@ -34673,10 +34653,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -35619,10 +35598,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>10</v>
+      </c>
+      <c r="E33" t="n">
+        <v>9</v>
+      </c>
+      <c r="F33" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="34">
@@ -35634,10 +35618,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>16</v>
+      </c>
+      <c r="E34" t="n">
+        <v>16</v>
+      </c>
+      <c r="F34" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="35">
@@ -35929,10 +35918,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>6</v>
+      </c>
+      <c r="E49" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="50">
@@ -37019,10 +37013,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>13</v>
+      </c>
+      <c r="E33" t="n">
+        <v>16</v>
+      </c>
+      <c r="F33" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="34">
@@ -37034,10 +37033,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>31</v>
+      </c>
+      <c r="E34" t="n">
+        <v>10</v>
+      </c>
+      <c r="F34" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="35">
@@ -37329,10 +37333,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>2</v>
+      </c>
+      <c r="E49" t="n">
+        <v>5</v>
+      </c>
+      <c r="F49" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="50">
@@ -38319,10 +38328,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="34">
@@ -38334,10 +38342,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="35">
@@ -38545,10 +38552,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="50">
@@ -39491,10 +39497,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>6</v>
+      </c>
+      <c r="E33" t="n">
+        <v>7</v>
+      </c>
+      <c r="F33" t="n">
+        <v>13</v>
       </c>
     </row>
     <row r="34">
@@ -39506,10 +39517,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>15</v>
+      </c>
+      <c r="E34" t="n">
+        <v>5</v>
+      </c>
+      <c r="F34" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="35">
@@ -39801,10 +39817,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>4</v>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -40791,10 +40812,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="34">
@@ -40806,10 +40826,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="35">
@@ -41017,10 +41036,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="50">
@@ -41863,10 +41881,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="34">
@@ -41878,10 +41895,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -42089,10 +42105,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="50">
@@ -42935,10 +42950,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="34">
@@ -42950,10 +42964,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="35">
@@ -43161,10 +43174,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="50">
@@ -44007,10 +44019,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="34">
@@ -44022,10 +44033,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="35">
@@ -44233,10 +44243,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="50">
@@ -45179,10 +45188,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>4</v>
+      </c>
+      <c r="E33" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="34">
@@ -45194,10 +45208,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>7</v>
+      </c>
+      <c r="E34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F34" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="35">
@@ -45489,10 +45508,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>6</v>
+      </c>
+      <c r="E49" t="n">
+        <v>5</v>
+      </c>
+      <c r="F49" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="50">
@@ -46579,10 +46603,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>27</v>
+      </c>
+      <c r="E33" t="n">
+        <v>36</v>
+      </c>
+      <c r="F33" t="n">
+        <v>63</v>
       </c>
     </row>
     <row r="34">
@@ -46594,10 +46623,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>29</v>
+      </c>
+      <c r="E34" t="n">
+        <v>52</v>
+      </c>
+      <c r="F34" t="n">
+        <v>81</v>
       </c>
     </row>
     <row r="35">
@@ -46889,10 +46923,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>8</v>
+      </c>
+      <c r="E49" t="n">
+        <v>6</v>
+      </c>
+      <c r="F49" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="50">
@@ -48017,10 +48056,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="34">
@@ -48032,10 +48070,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="35">
@@ -48243,10 +48280,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="50">
@@ -49089,10 +49125,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="34">
@@ -49104,10 +49139,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="35">
@@ -49315,10 +49349,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -50161,10 +50194,9 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>37</v>
       </c>
     </row>
     <row r="34">
@@ -50176,10 +50208,9 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="35">
@@ -50387,10 +50418,9 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="50">
@@ -51333,10 +51363,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>7</v>
+      </c>
+      <c r="E33" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="34">
@@ -51348,10 +51383,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>7</v>
+      </c>
+      <c r="E34" t="n">
+        <v>22</v>
+      </c>
+      <c r="F34" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="35">
@@ -51643,10 +51683,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>3</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2</v>
+      </c>
+      <c r="F49" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="50">
@@ -52733,10 +52778,15 @@
           <t>08:00</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="n">
+        <v>2</v>
+      </c>
+      <c r="F33" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="34">
@@ -52748,10 +52798,15 @@
           <t>09:00</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>9</v>
+      </c>
+      <c r="E34" t="n">
+        <v>11</v>
+      </c>
+      <c r="F34" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="35">
@@ -53043,10 +53098,15 @@
           <t>24:00</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>zastarelo</t>
-        </is>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="50">

</xml_diff>

<commit_message>
Izlaz u formatu istorijskog mastera (y_A, razlog_A) i Excel kolona y_A umesto S
- satno.py: podaci/YYYY/MM/master_YYYY-MM.parquet — stanica_id, ts, y_A, razlog_A (+ datum, sat),
  puna naivna satna mreza; DST kao master (jesen: prvi od dva ista ts, prolece: nema_reda); --spoji
  pravi i podaci/master_novo.parquet
- excel.py: serija sa jednim smerom ima kolonu y_A (cilj modela, istorijski A1k/A2k), ne S<n>
- testovi za master format na danima prelaska vremena

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HjLihUGrpExWnzAPATqsnz
</commit_message>
<xml_diff>
--- a/podaci/excel/bicikli_2026-10.xlsx
+++ b/podaci/excel/bicikli_2026-10.xlsx
@@ -524,7 +524,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -1609,7 +1609,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -5434,7 +5434,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -7604,7 +7604,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -8689,7 +8689,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9774,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -10859,7 +10859,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -11944,7 +11944,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -13029,7 +13029,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -14114,7 +14114,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -15199,7 +15199,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -16296,7 +16296,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -17381,7 +17381,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -18466,7 +18466,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -19551,7 +19551,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -20636,7 +20636,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -26110,7 +26110,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -27195,7 +27195,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -28404,7 +28404,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -29489,7 +29489,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -30574,7 +30574,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -31659,7 +31659,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -32744,7 +32744,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -33829,7 +33829,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -34914,7 +34914,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -38925,7 +38925,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -41473,7 +41473,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -42558,7 +42558,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -43739,7 +43739,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -44824,7 +44824,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -48810,7 +48810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -48844,154 +48844,166 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>S&lt;n&gt; / Sum1, Sum2</t>
+          <t>y_A</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>broj biciklista po smeru; Sum = zbir smerova (samo kada oba smera imaju vrednost)</t>
+          <t>broj biciklista (cilj modela) — serija sa jednim smerom</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Status prazan</t>
+          <t>Sum1, Sum2, Sum</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>sat je ispravan</t>
+          <t>stari dvosmerni brojači: po smeru i zbir (Sum = y_A, samo kada oba smera imaju vrednost)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>nema_citanja</t>
+          <t>Status prazan</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>čitanje u tom satu nije uspelo</t>
+          <t>sat je ispravan</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nema_smera</t>
+          <t>nema_citanja</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>u čitanju nema tog smera</t>
+          <t>čitanje u tom satu nije uspelo</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>zastarelo</t>
+          <t>nema_smera</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>podatak brojača je prestar (uređaj ne javlja nove podatke)</t>
+          <t>u čitanju nema tog smera</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>nepotpun_sat</t>
+          <t>zastarelo</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>razmak čitanja nije ~1 sat</t>
+          <t>podatak brojača je prestar (uređaj ne javlja nove podatke)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>negativna_razlika</t>
+          <t>nepotpun_sat</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>brojač je resetovan</t>
+          <t>razmak čitanja nije ~1 sat</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Crveno</t>
+          <t>negativna_razlika</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>vrednost &gt; 400</t>
+          <t>brojač je resetovan</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sivo</t>
+          <t>Crveno</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>nema vrednosti za taj sat (razlog u Status)</t>
+          <t>vrednost &gt; 400</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Narandžasto: nula_dan</t>
+          <t>Sivo</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>smer je ceo dan imao 0 biciklista (moguće neispravan senzor)</t>
+          <t>nema vrednosti za taj sat (razlog u Status)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Narandžasto: nula_niz</t>
+          <t>Narandžasto: nula_dan</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>≥ 3 uzastopna sata sa 0 između 07:00 i 21:00, a smer tog dana ima ≥ 100</t>
+          <t>smer je ceo dan imao 0 biciklista (moguće neispravan senzor)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Žuto: skok</t>
+          <t>Narandžasto: nula_niz</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>vrednost ≥ 50 i ≥ 3× veća od oba susedna sata</t>
+          <t>≥ 3 uzastopna sata sa 0 između 07:00 i 21:00, a smer tog dana ima ≥ 100</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Žuto: skok</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>vrednost ≥ 50 i ≥ 3× veća od oba susedna sata</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Napomena</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>markirane vrednosti NISU menjane — markiranje samo upozorava; odluka je na korisniku</t>
         </is>
@@ -49033,7 +49045,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -50118,7 +50130,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S3</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>
@@ -51203,7 +51215,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>S4</t>
+          <t>y_A</t>
         </is>
       </c>
     </row>

</xml_diff>